<commit_message>
ajout de la sauvegarde
</commit_message>
<xml_diff>
--- a/Projet Le Solitaire 2026 (auto-évaluation _ soutenances).xlsx
+++ b/Projet Le Solitaire 2026 (auto-évaluation _ soutenances).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Devoirs\projet python solitaire\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87008696-1EF8-4B0F-AFAC-8B5D2A67AF6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4E45362-6C6B-464D-B7F5-A2A4EF34E265}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -75,7 +75,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="67">
   <si>
     <t>Soutenances du projet - Le Solitaire</t>
   </si>
@@ -294,6 +294,12 @@
   <si>
     <t>ctypes</t>
   </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>json</t>
+  </si>
 </sst>
 </file>
 
@@ -430,7 +436,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -520,6 +526,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="10" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1117,7 +1126,7 @@
       <c r="AP4" s="15"/>
     </row>
     <row r="5" spans="1:42" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="34" t="s">
         <v>22</v>
       </c>
       <c r="B5" s="17"/>
@@ -1264,7 +1273,7 @@
       </c>
       <c r="B8" s="15"/>
       <c r="C8" s="20" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D8" s="15"/>
       <c r="E8" s="15"/>
@@ -1360,7 +1369,7 @@
       </c>
       <c r="B10" s="15"/>
       <c r="C10" s="20" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D10" s="15"/>
       <c r="E10" s="15"/>
@@ -2072,7 +2081,7 @@
       </c>
       <c r="B25" s="15"/>
       <c r="C25" s="20" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D25" s="15"/>
       <c r="E25" s="15"/>
@@ -2218,7 +2227,7 @@
       </c>
       <c r="B28" s="15"/>
       <c r="C28" s="20" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D28" s="15"/>
       <c r="E28" s="15"/>
@@ -2687,7 +2696,9 @@
     <row r="38" spans="1:42" ht="13.8" x14ac:dyDescent="0.3">
       <c r="A38" s="26"/>
       <c r="B38" s="15"/>
-      <c r="C38" s="20"/>
+      <c r="C38" s="20" t="s">
+        <v>66</v>
+      </c>
       <c r="D38" s="15"/>
       <c r="E38" s="15"/>
       <c r="F38" s="15"/>

</xml_diff>

<commit_message>
ajout du déplacement d'une fondation vers une colonne
</commit_message>
<xml_diff>
--- a/Projet Le Solitaire 2026 (auto-évaluation _ soutenances).xlsx
+++ b/Projet Le Solitaire 2026 (auto-évaluation _ soutenances).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Devoirs\projet python solitaire\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4E45362-6C6B-464D-B7F5-A2A4EF34E265}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{040F5365-B7D5-461B-93D2-42E9276ECDB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -75,7 +75,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="66">
   <si>
     <t>Soutenances du projet - Le Solitaire</t>
   </si>
@@ -293,9 +293,6 @@
   </si>
   <si>
     <t>ctypes</t>
-  </si>
-  <si>
-    <t>In Progress</t>
   </si>
   <si>
     <t>json</t>
@@ -2081,7 +2078,7 @@
       </c>
       <c r="B25" s="15"/>
       <c r="C25" s="20" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="D25" s="15"/>
       <c r="E25" s="15"/>
@@ -2131,7 +2128,7 @@
         <v>44</v>
       </c>
       <c r="C26" s="20" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D26" s="15"/>
       <c r="E26" s="15"/>
@@ -2697,7 +2694,7 @@
       <c r="A38" s="26"/>
       <c r="B38" s="15"/>
       <c r="C38" s="20" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D38" s="15"/>
       <c r="E38" s="15"/>

</xml_diff>